<commit_message>
Milestone - all scripts and functionality working. To this point.
</commit_message>
<xml_diff>
--- a/database/series_setup.xlsx
+++ b/database/series_setup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Series" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
   <si>
     <t>Name</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t>Stage X</t>
+  </si>
+  <si>
+    <t>b02d01d1-d21e-4095-8788-878691be5de9</t>
+  </si>
+  <si>
+    <t>a880966a-1325-4a1d-882a-ece2dcbf9244</t>
   </si>
 </sst>
 </file>
@@ -774,7 +780,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.77734375" bestFit="1" customWidth="1"/>
@@ -801,6 +807,16 @@
         <v>28</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>